<commit_message>
adds two new handlers to the garage
</commit_message>
<xml_diff>
--- a/HealthcareSolutions.suite/Resources/HDREG-1.xlsx
+++ b/HealthcareSolutions.suite/Resources/HDREG-1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26827"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="libxl" lastEdited="7" lowestEdited="7" rupBuild="4.6.0"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ScriptRepositories\HealthcareSolutions\HealthcareSolutions.suite\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FF73597-BB71-4763-B9BF-B7438D1C45D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA65CC02-01B5-4CE8-9130-01D28773AFC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100"/>
   </bookViews>
   <sheets>
     <sheet name="Current" sheetId="1" r:id="rId1"/>
@@ -18,9 +18,9 @@
     <sheet name="New" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">New!$A$1:$AK$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="true">New!$A$1:$AK$124</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="true"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>tc={9DDA84F1-6010-4F5F-BF85-B64D39570119}</author>
     <author>tc={7B6D4E81-E186-4946-A759-D0DD3316DAB3}</author>
@@ -71,7 +71,7 @@
     <author>tc={756156C0-60AF-485B-BF15-02831CFD22D0}</author>
   </authors>
   <commentList>
-    <comment ref="W1" authorId="0" shapeId="0" xr:uid="{9DDA84F1-6010-4F5F-BF85-B64D39570119}">
+    <comment ref="W1" authorId="0">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -79,7 +79,7 @@
     EPT 145</t>
       </text>
     </comment>
-    <comment ref="P2" authorId="1" shapeId="0" xr:uid="{7B6D4E81-E186-4946-A759-D0DD3316DAB3}">
+    <comment ref="P2" authorId="1">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -87,7 +87,7 @@
     Single</t>
       </text>
     </comment>
-    <comment ref="Q2" authorId="2" shapeId="0" xr:uid="{998F6731-21B5-4536-905C-40876AE868A8}">
+    <comment ref="Q2" authorId="2">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -95,7 +95,7 @@
     US Citizen</t>
       </text>
     </comment>
-    <comment ref="V2" authorId="3" shapeId="0" xr:uid="{E7489066-7AF8-4C7C-8270-4F0F00088EBD}">
+    <comment ref="V2" authorId="3">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -103,7 +103,7 @@
     Not hispanic</t>
       </text>
     </comment>
-    <comment ref="Q3" authorId="4" shapeId="0" xr:uid="{26FF9C4A-AA48-48D1-96CD-D4D2583FF86A}">
+    <comment ref="Q3" authorId="4">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -111,7 +111,7 @@
     Non-US Citizen</t>
       </text>
     </comment>
-    <comment ref="V3" authorId="5" shapeId="0" xr:uid="{4836FEDC-8B37-4192-8F1B-A6B769869267}">
+    <comment ref="V3" authorId="5">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -119,7 +119,7 @@
     Unknown</t>
       </text>
     </comment>
-    <comment ref="P4" authorId="6" shapeId="0" xr:uid="{30BA3AAE-5D1C-4297-8E46-309621332630}">
+    <comment ref="P4" authorId="6">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -127,7 +127,7 @@
     Married</t>
       </text>
     </comment>
-    <comment ref="Q4" authorId="7" shapeId="0" xr:uid="{5011934E-75E1-4902-A395-288719F42165}">
+    <comment ref="Q4" authorId="7">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -135,7 +135,7 @@
     Foreign US Resident</t>
       </text>
     </comment>
-    <comment ref="R4" authorId="8" shapeId="0" xr:uid="{DBAA2B4C-E086-47EF-9044-30637FAC5623}">
+    <comment ref="R4" authorId="8">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -143,7 +143,7 @@
     Yes, separated</t>
       </text>
     </comment>
-    <comment ref="V4" authorId="9" shapeId="0" xr:uid="{D89D251D-F0E8-4C73-9700-C3DA24906A09}">
+    <comment ref="V4" authorId="9">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -151,7 +151,7 @@
     Decline</t>
       </text>
     </comment>
-    <comment ref="Q5" authorId="10" shapeId="0" xr:uid="{9AA9ADB8-3732-48AB-8A32-496E2C650879}">
+    <comment ref="Q5" authorId="10">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -159,7 +159,7 @@
     US Resident</t>
       </text>
     </comment>
-    <comment ref="R5" authorId="11" shapeId="0" xr:uid="{5C2A6ACB-D6F4-4340-828E-C4C9ED1A5DBE}">
+    <comment ref="R5" authorId="11">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -167,7 +167,7 @@
     No, never served</t>
       </text>
     </comment>
-    <comment ref="V5" authorId="12" shapeId="0" xr:uid="{343D88B6-4637-47BD-83A8-3C14B2AEAA44}">
+    <comment ref="V5" authorId="12">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -175,7 +175,7 @@
     Mexican</t>
       </text>
     </comment>
-    <comment ref="P6" authorId="13" shapeId="0" xr:uid="{33F2BB15-5B81-4FB4-8494-3482D7DDC8CE}">
+    <comment ref="P6" authorId="13">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -183,7 +183,7 @@
     Legally separated</t>
       </text>
     </comment>
-    <comment ref="R6" authorId="14" shapeId="0" xr:uid="{B883C31E-51BD-494F-AC12-05387E3490F4}">
+    <comment ref="R6" authorId="14">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -191,7 +191,7 @@
     Yes, separated/combat veteran</t>
       </text>
     </comment>
-    <comment ref="V6" authorId="15" shapeId="0" xr:uid="{2B563F96-60E3-4BE1-AB58-5D7520E2CC0E}">
+    <comment ref="V6" authorId="15">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -199,7 +199,7 @@
     Puerto Rican</t>
       </text>
     </comment>
-    <comment ref="P7" authorId="16" shapeId="0" xr:uid="{3D2865E7-B550-481A-8044-5EFFEA88F4BA}">
+    <comment ref="P7" authorId="16">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -207,7 +207,7 @@
     Divorced</t>
       </text>
     </comment>
-    <comment ref="R7" authorId="17" shapeId="0" xr:uid="{F6DE0FEA-2B03-43B6-8EB2-635106A4882F}">
+    <comment ref="R7" authorId="17">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -215,7 +215,7 @@
     Declined</t>
       </text>
     </comment>
-    <comment ref="V7" authorId="18" shapeId="0" xr:uid="{766DD95C-1DA8-40BC-9298-EFA08E7DA978}">
+    <comment ref="V7" authorId="18">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -223,7 +223,7 @@
     Cuban</t>
       </text>
     </comment>
-    <comment ref="P8" authorId="19" shapeId="0" xr:uid="{7501C7B3-C1D5-494F-BEFE-553F3876D663}">
+    <comment ref="P8" authorId="19">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -231,7 +231,7 @@
     Widowed</t>
       </text>
     </comment>
-    <comment ref="R8" authorId="20" shapeId="0" xr:uid="{61A6A439-749E-415C-AB57-3FE4F216606F}">
+    <comment ref="R8" authorId="20">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -239,7 +239,7 @@
     Yes, Currently serving</t>
       </text>
     </comment>
-    <comment ref="V8" authorId="21" shapeId="0" xr:uid="{0DF6E6D2-895E-48B1-BB16-F68E00A73043}">
+    <comment ref="V8" authorId="21">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -247,7 +247,7 @@
     Hispanic</t>
       </text>
     </comment>
-    <comment ref="P9" authorId="22" shapeId="0" xr:uid="{71BFB5F2-B03D-4DB1-9AEB-FEF1317C6AD5}">
+    <comment ref="P9" authorId="22">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -255,7 +255,7 @@
     Unknown</t>
       </text>
     </comment>
-    <comment ref="R9" authorId="23" shapeId="0" xr:uid="{541C595E-FEFA-45EA-A3DE-0D6D5B71ECE3}">
+    <comment ref="R9" authorId="23">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -263,7 +263,7 @@
     No, currently serving</t>
       </text>
     </comment>
-    <comment ref="P10" authorId="24" shapeId="0" xr:uid="{29E9E735-0A37-49CB-A1CE-186C078976D2}">
+    <comment ref="P10" authorId="24">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -271,7 +271,7 @@
     Significant Other</t>
       </text>
     </comment>
-    <comment ref="P11" authorId="25" shapeId="0" xr:uid="{756156C0-60AF-485B-BF15-02831CFD22D0}">
+    <comment ref="P11" authorId="25">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -284,7 +284,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1750" uniqueCount="422">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="1751" uniqueCount="423">
   <si>
     <t>RecNumber</t>
   </si>
@@ -1550,13 +1550,16 @@
   </si>
   <si>
     <t>361636</t>
+  </si>
+  <si>
+    <t>Eggplant, Aidan</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1595,7 +1598,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
+        <fgColor theme="9" tint="0.39997558519242"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1621,17 +1624,17 @@
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="true" applyFill="true"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 119" xfId="1" xr:uid="{48203254-307B-4614-938C-E53FFE43CCEC}"/>
+    <cellStyle name="Normal 119" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1658,9 +1661,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1698,7 +1701,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1804,12 +1807,12 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1833,9 +1836,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1859,7 +1862,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1894,7 +1897,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -1912,7 +1915,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1937,7 +1940,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -1946,7 +1949,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2036,62 +2039,62 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AZ45"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.61328125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.61328125" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.69140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.53515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.07421875" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.84375" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="7" style="3" customWidth="1"/>
-    <col min="11" max="11" width="9.84375" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.3046875" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.53515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.07421875" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.15234375" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.4609375" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15.23046875" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.69140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.3046875" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.07421875" style="3" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.765625" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.61328125" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="33.07421875" style="3" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="13.23046875" style="3" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="16.84375" style="3" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="7.4609375" style="3" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="19.53515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="8.07421875" style="3" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="13.84375" style="3" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="4.84375" style="3" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="32.61328125" style="3" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="6.69140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="21.53515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="27" style="3" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="21.23046875" style="3" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="19.921875" style="3" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="14.765625" style="3" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="22.765625" style="3" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="26.4609375" style="3" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="17.4609375" style="3" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="25.4609375" style="3" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="26.4609375" style="3" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="17.61328125" style="3" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="12.53515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="15.84375" style="3" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="21.15234375" style="3" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="21.15234375" style="3" customWidth="1"/>
-    <col min="51" max="51" width="23.84375" style="3" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="6.921875" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.6328125" style="3" bestFit="true" customWidth="true"/>
+    <col min="2" max="2" width="10.6328125" style="5" bestFit="true" customWidth="true"/>
+    <col min="3" max="3" width="18.7265625" style="3" bestFit="true" customWidth="true"/>
+    <col min="4" max="4" width="10.54296875" style="3" bestFit="true" customWidth="true"/>
+    <col min="5" max="5" width="9.08984375" style="3" bestFit="true" customWidth="true"/>
+    <col min="6" max="6" width="8.81640625" style="3" bestFit="true" customWidth="true"/>
+    <col min="7" max="7" width="7" style="3" bestFit="true" customWidth="true"/>
+    <col min="8" max="10" width="7" style="3" customWidth="true"/>
+    <col min="11" max="11" width="9.81640625" style="3" bestFit="true" customWidth="true"/>
+    <col min="12" max="12" width="17.26953125" style="3" bestFit="true" customWidth="true"/>
+    <col min="13" max="13" width="7.54296875" style="3" bestFit="true" customWidth="true"/>
+    <col min="14" max="14" width="11.08984375" style="3" bestFit="true" customWidth="true"/>
+    <col min="15" max="15" width="12" style="3" bestFit="true" customWidth="true"/>
+    <col min="16" max="16" width="21.1796875" style="3" bestFit="true" customWidth="true"/>
+    <col min="17" max="17" width="14.453125" style="3" bestFit="true" customWidth="true"/>
+    <col min="18" max="18" width="15.26953125" style="3" bestFit="true" customWidth="true"/>
+    <col min="19" max="19" width="8.7265625" style="3" bestFit="true" customWidth="true"/>
+    <col min="20" max="20" width="12.26953125" style="3" bestFit="true" customWidth="true"/>
+    <col min="21" max="21" width="12.08984375" style="3" bestFit="true" customWidth="true"/>
+    <col min="22" max="22" width="15.7265625" style="3" bestFit="true" customWidth="true"/>
+    <col min="23" max="23" width="12.6328125" style="3" bestFit="true" customWidth="true"/>
+    <col min="24" max="24" width="33.08984375" style="3" bestFit="true" customWidth="true"/>
+    <col min="25" max="25" width="13.26953125" style="3" bestFit="true" customWidth="true"/>
+    <col min="26" max="26" width="16.81640625" style="3" bestFit="true" customWidth="true"/>
+    <col min="27" max="27" width="7.453125" style="3" bestFit="true" customWidth="true"/>
+    <col min="28" max="28" width="19.54296875" style="3" bestFit="true" customWidth="true"/>
+    <col min="29" max="29" width="8.08984375" style="3" bestFit="true" customWidth="true"/>
+    <col min="30" max="30" width="13.81640625" style="3" bestFit="true" customWidth="true"/>
+    <col min="31" max="31" width="4.81640625" style="3" bestFit="true" customWidth="true"/>
+    <col min="32" max="32" width="32.6328125" style="3" bestFit="true" customWidth="true"/>
+    <col min="33" max="33" width="6.7265625" style="3" bestFit="true" customWidth="true"/>
+    <col min="34" max="34" width="21.54296875" style="3" bestFit="true" customWidth="true"/>
+    <col min="35" max="36" width="27" style="3" bestFit="true" customWidth="true"/>
+    <col min="37" max="37" width="21.26953125" style="3" bestFit="true" customWidth="true"/>
+    <col min="38" max="38" width="19.90625" style="3" bestFit="true" customWidth="true"/>
+    <col min="39" max="39" width="14.7265625" style="3" bestFit="true" customWidth="true"/>
+    <col min="40" max="40" width="22.7265625" style="3" bestFit="true" customWidth="true"/>
+    <col min="41" max="41" width="26.453125" style="3" bestFit="true" customWidth="true"/>
+    <col min="42" max="42" width="17.453125" style="3" bestFit="true" customWidth="true"/>
+    <col min="43" max="43" width="25.453125" style="3" bestFit="true" customWidth="true"/>
+    <col min="44" max="44" width="26.453125" style="3" bestFit="true" customWidth="true"/>
+    <col min="45" max="45" width="17.6328125" style="3" bestFit="true" customWidth="true"/>
+    <col min="46" max="46" width="12.54296875" style="3" bestFit="true" customWidth="true"/>
+    <col min="47" max="47" width="15.81640625" style="3" bestFit="true" customWidth="true"/>
+    <col min="48" max="48" width="13" style="3" bestFit="true" customWidth="true"/>
+    <col min="49" max="49" width="21.1796875" style="3" bestFit="true" customWidth="true"/>
+    <col min="50" max="50" width="21.1796875" style="3" customWidth="true"/>
+    <col min="51" max="51" width="23.81640625" style="3" bestFit="true" customWidth="true"/>
+    <col min="52" max="52" width="6.90625" style="5" bestFit="true" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" s="1" customFormat="true" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2249,16 +2252,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:52" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>421</v>
       </c>
-      <c r="C2" s="3" t="str">
-        <f t="shared" ref="C2:C32" si="0">CONCATENATE(E2,", ",D2)</f>
-        <v>Eggplant, Alden</v>
+      <c r="C2" s="3" t="s">
+        <v>422</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>329</v>
@@ -2400,12 +2402,12 @@
         <v>272</v>
       </c>
     </row>
-    <row r="3" spans="1:52" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="C3" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="C2:C32" si="0">CONCATENATE(E3,", ",D3)</f>
         <v>Eggplant, Sophia</v>
       </c>
       <c r="D3" s="3" t="s">
@@ -2484,7 +2486,7 @@
         <v>228</v>
       </c>
       <c r="AC3" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AD3" s="3" t="s">
         <v>352</v>
@@ -2551,7 +2553,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="4" spans="1:52" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -2696,7 +2698,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="5" spans="1:52" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -2847,7 +2849,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="6" spans="1:52" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -2988,7 +2990,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="7" spans="1:52" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -3129,7 +3131,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="8" spans="1:52" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -3276,7 +3278,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="9" spans="1:52" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -3423,7 +3425,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="10" spans="1:52" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -3570,7 +3572,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:52" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -3717,7 +3719,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:52" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -3865,7 +3867,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:52" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -4012,7 +4014,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:52" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -4160,7 +4162,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:52" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -4311,7 +4313,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:52" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -4468,7 +4470,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:51" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -4613,7 +4615,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="18" spans="1:51" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -4764,7 +4766,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="19" spans="1:51" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -4909,7 +4911,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="20" spans="1:51" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -5060,7 +5062,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="21" spans="1:51" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -5205,7 +5207,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="22" spans="1:51" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -5356,7 +5358,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="23" spans="1:51" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -5501,7 +5503,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="24" spans="1:51" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -5652,7 +5654,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="25" spans="1:51" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -5797,7 +5799,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="26" spans="1:51" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -5948,7 +5950,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="27" spans="1:51" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -6051,7 +6053,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="28" spans="1:51" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -6136,7 +6138,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="29" spans="1:51" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -6221,7 +6223,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="30" spans="1:51" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -6306,7 +6308,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="31" spans="1:51" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -6391,7 +6393,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="32" spans="1:51" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -6476,7 +6478,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="33" spans="1:44" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="33" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -6561,7 +6563,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="34" spans="1:44" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" x14ac:dyDescent="0.35">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -6646,7 +6648,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="35" spans="1:44" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="35" x14ac:dyDescent="0.35">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -6731,7 +6733,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="36" spans="1:44" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="36" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -6816,7 +6818,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="37" spans="1:44" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="37" x14ac:dyDescent="0.35">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -6901,7 +6903,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="38" spans="1:44" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="38" x14ac:dyDescent="0.35">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -6986,7 +6988,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="39" spans="1:44" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="39" x14ac:dyDescent="0.35">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -7071,7 +7073,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="40" spans="1:44" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="40" x14ac:dyDescent="0.35">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -7156,7 +7158,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="41" spans="1:44" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="41" x14ac:dyDescent="0.35">
       <c r="A41" s="3">
         <v>40</v>
       </c>
@@ -7241,7 +7243,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="42" spans="1:44" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="42" x14ac:dyDescent="0.35">
       <c r="A42" s="3">
         <v>41</v>
       </c>
@@ -7326,7 +7328,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="43" spans="1:44" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="43" x14ac:dyDescent="0.35">
       <c r="A43" s="3">
         <v>42</v>
       </c>
@@ -7411,7 +7413,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="44" spans="1:44" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="44" x14ac:dyDescent="0.35">
       <c r="A44" s="3">
         <v>43</v>
       </c>
@@ -7496,7 +7498,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="45" spans="1:44" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="45" x14ac:dyDescent="0.35">
       <c r="A45" s="3">
         <v>44</v>
       </c>
@@ -7589,9 +7591,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34DBB9F2-8D7A-4165-961E-4CD41274F703}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34DBB9F2-8D7A-4165-961E-4CD41274F703}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7600,48 +7602,48 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2701B23F-DA41-4F48-B4AF-4C926B2F5894}">
   <dimension ref="A1:AK124"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.3828125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.69140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.61328125" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.23046875" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.921875" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.69140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.921875" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.69140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.15234375" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.53515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.921875" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.84375" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.15234375" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.07421875" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.23046875" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.84375" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.3828125" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.4609375" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.3046875" style="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="21.15234375" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="18.3828125" style="3" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="26.84375" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="2.69140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="6.07421875" style="3" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="23.07421875" style="3" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="28.4609375" style="3" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="20" style="3" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="21.53515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="16.53515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="24.3828125" style="3" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="19.07421875" style="3" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="26.84375" style="3" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="22.53515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="14.3046875" style="3" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="12.53515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="8.765625" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.36328125" style="3" bestFit="true" customWidth="true"/>
+    <col min="2" max="2" width="9.7265625" style="5" bestFit="true" customWidth="true"/>
+    <col min="3" max="3" width="17.6328125" style="3" bestFit="true" customWidth="true"/>
+    <col min="4" max="4" width="11.26953125" style="3" bestFit="true" customWidth="true"/>
+    <col min="5" max="5" width="10.90625" style="3" bestFit="true" customWidth="true"/>
+    <col min="6" max="6" width="8.7265625" style="3" bestFit="true" customWidth="true"/>
+    <col min="7" max="7" width="8.90625" style="3" bestFit="true" customWidth="true"/>
+    <col min="8" max="8" width="9.7265625" style="3" bestFit="true" customWidth="true"/>
+    <col min="9" max="9" width="14.1796875" style="3" bestFit="true" customWidth="true"/>
+    <col min="10" max="10" width="9.54296875" style="3" bestFit="true" customWidth="true"/>
+    <col min="11" max="11" width="12.90625" style="3" bestFit="true" customWidth="true"/>
+    <col min="12" max="12" width="13.81640625" style="3" bestFit="true" customWidth="true"/>
+    <col min="13" max="13" width="20.1796875" style="3" bestFit="true" customWidth="true"/>
+    <col min="14" max="14" width="17.08984375" style="3" bestFit="true" customWidth="true"/>
+    <col min="15" max="15" width="16.26953125" style="3" bestFit="true" customWidth="true"/>
+    <col min="16" max="16" width="13.81640625" style="3" bestFit="true" customWidth="true"/>
+    <col min="17" max="17" width="8.36328125" style="3" bestFit="true" customWidth="true"/>
+    <col min="18" max="18" width="14.453125" style="3" bestFit="true" customWidth="true"/>
+    <col min="19" max="19" width="16.26953125" style="3" bestFit="true" customWidth="true"/>
+    <col min="20" max="20" width="21.1796875" style="3" bestFit="true" customWidth="true"/>
+    <col min="21" max="21" width="18.36328125" style="3" bestFit="true" customWidth="true"/>
+    <col min="22" max="22" width="10" style="3" bestFit="true" customWidth="true"/>
+    <col min="23" max="23" width="26.81640625" style="3" bestFit="true" customWidth="true"/>
+    <col min="24" max="24" width="2.7265625" style="3" bestFit="true" customWidth="true"/>
+    <col min="25" max="25" width="6.08984375" style="3" bestFit="true" customWidth="true"/>
+    <col min="26" max="26" width="23.08984375" style="3" bestFit="true" customWidth="true"/>
+    <col min="27" max="27" width="28.453125" style="3" bestFit="true" customWidth="true"/>
+    <col min="28" max="28" width="20" style="3" bestFit="true" customWidth="true"/>
+    <col min="29" max="29" width="21.54296875" style="3" bestFit="true" customWidth="true"/>
+    <col min="30" max="30" width="16.54296875" style="3" bestFit="true" customWidth="true"/>
+    <col min="31" max="31" width="24.36328125" style="3" bestFit="true" customWidth="true"/>
+    <col min="32" max="32" width="19.08984375" style="3" bestFit="true" customWidth="true"/>
+    <col min="33" max="33" width="26.81640625" style="3" bestFit="true" customWidth="true"/>
+    <col min="34" max="34" width="22.54296875" style="3" bestFit="true" customWidth="true"/>
+    <col min="35" max="35" width="14.26953125" style="3" bestFit="true" customWidth="true"/>
+    <col min="36" max="36" width="12.54296875" style="3" bestFit="true" customWidth="true"/>
+    <col min="37" max="37" width="8.7265625" style="5" bestFit="true" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" s="1" customFormat="true" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -7752,7 +7754,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -7845,7 +7847,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -7941,7 +7943,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -8055,7 +8057,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -8151,7 +8153,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -8265,7 +8267,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -8364,7 +8366,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="8" spans="1:37" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -8460,7 +8462,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="9" spans="1:37" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -8550,7 +8552,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -8640,7 +8642,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -8715,7 +8717,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -8785,7 +8787,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -8854,7 +8856,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -8909,7 +8911,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -8963,7 +8965,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:37" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -9017,7 +9019,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -9071,7 +9073,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -9119,7 +9121,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -9161,7 +9163,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -9203,7 +9205,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -9245,7 +9247,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -9287,7 +9289,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="23" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -9329,7 +9331,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -9380,7 +9382,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="25" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -9431,7 +9433,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="26" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -9482,7 +9484,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="27" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -9533,7 +9535,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="28" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -9593,7 +9595,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="29" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -9653,7 +9655,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="30" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -9713,7 +9715,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="31" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -9773,7 +9775,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="32" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -9833,7 +9835,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="33" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="33" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -9893,7 +9895,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="34" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" x14ac:dyDescent="0.35">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -9953,7 +9955,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="35" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="35" x14ac:dyDescent="0.35">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -10013,7 +10015,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="36" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="36" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -10073,7 +10075,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="37" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="37" x14ac:dyDescent="0.35">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -10133,7 +10135,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="38" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="38" x14ac:dyDescent="0.35">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -10190,7 +10192,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="39" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="39" x14ac:dyDescent="0.35">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -10247,7 +10249,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="40" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="40" x14ac:dyDescent="0.35">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -10304,7 +10306,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="41" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="41" x14ac:dyDescent="0.35">
       <c r="A41" s="3">
         <v>40</v>
       </c>
@@ -10361,7 +10363,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="42" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="42" x14ac:dyDescent="0.35">
       <c r="A42" s="3">
         <v>41</v>
       </c>
@@ -10418,7 +10420,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="43" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="43" x14ac:dyDescent="0.35">
       <c r="A43" s="3">
         <v>42</v>
       </c>
@@ -10475,7 +10477,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="44" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="44" x14ac:dyDescent="0.35">
       <c r="A44" s="3">
         <v>43</v>
       </c>
@@ -10532,7 +10534,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="45" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="45" x14ac:dyDescent="0.35">
       <c r="A45" s="3">
         <v>44</v>
       </c>
@@ -10589,7 +10591,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="46" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="46" x14ac:dyDescent="0.35">
       <c r="N46" s="3" t="s">
         <v>32</v>
       </c>
@@ -10597,7 +10599,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="47" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="47" x14ac:dyDescent="0.35">
       <c r="N47" s="3" t="s">
         <v>93</v>
       </c>
@@ -10605,7 +10607,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="48" spans="1:36" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="48" x14ac:dyDescent="0.35">
       <c r="N48" s="3" t="s">
         <v>32</v>
       </c>
@@ -10613,7 +10615,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="49" spans="14:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="49" x14ac:dyDescent="0.35">
       <c r="N49" s="3" t="s">
         <v>93</v>
       </c>
@@ -10621,383 +10623,383 @@
         <v>155</v>
       </c>
     </row>
-    <row r="50" spans="14:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="50" x14ac:dyDescent="0.35">
       <c r="O50" s="3" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="51" spans="14:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="51" x14ac:dyDescent="0.35">
       <c r="O51" s="3" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="52" spans="14:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="52" x14ac:dyDescent="0.35">
       <c r="O52" s="3" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="53" spans="14:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="53" x14ac:dyDescent="0.35">
       <c r="O53" s="3" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="54" spans="14:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="54" x14ac:dyDescent="0.35">
       <c r="O54" s="3" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="55" spans="14:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="55" x14ac:dyDescent="0.35">
       <c r="O55" s="3" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="56" spans="14:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="56" x14ac:dyDescent="0.35">
       <c r="O56" s="3" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="57" spans="14:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="57" x14ac:dyDescent="0.35">
       <c r="O57" s="3" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="58" spans="14:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="58" x14ac:dyDescent="0.35">
       <c r="O58" s="3" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="59" spans="14:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="59" x14ac:dyDescent="0.35">
       <c r="O59" s="3" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="60" spans="14:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="60" x14ac:dyDescent="0.35">
       <c r="O60" s="3" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="61" spans="14:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="61" x14ac:dyDescent="0.35">
       <c r="O61" s="3" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="62" spans="14:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="62" x14ac:dyDescent="0.35">
       <c r="O62" s="3" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="63" spans="14:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="63" x14ac:dyDescent="0.35">
       <c r="O63" s="3" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="64" spans="14:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="64" x14ac:dyDescent="0.35">
       <c r="O64" s="3" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="65" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="65" x14ac:dyDescent="0.35">
       <c r="O65" s="3" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="66" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="66" x14ac:dyDescent="0.35">
       <c r="O66" s="3" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="67" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="67" x14ac:dyDescent="0.35">
       <c r="O67" s="3" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="68" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="68" x14ac:dyDescent="0.35">
       <c r="O68" s="3" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="69" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="69" x14ac:dyDescent="0.35">
       <c r="O69" s="3" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="70" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="70" x14ac:dyDescent="0.35">
       <c r="O70" s="3" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="71" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="71" x14ac:dyDescent="0.35">
       <c r="O71" s="3" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="72" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="72" x14ac:dyDescent="0.35">
       <c r="O72" s="3" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="73" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="73" x14ac:dyDescent="0.35">
       <c r="O73" s="3" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="74" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="74" x14ac:dyDescent="0.35">
       <c r="O74" s="3" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="75" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="75" x14ac:dyDescent="0.35">
       <c r="O75" s="3" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="76" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="76" x14ac:dyDescent="0.35">
       <c r="O76" s="3" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="77" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="77" x14ac:dyDescent="0.35">
       <c r="O77" s="3" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="78" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="78" x14ac:dyDescent="0.35">
       <c r="O78" s="3" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="79" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="79" x14ac:dyDescent="0.35">
       <c r="O79" s="3" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="80" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="80" x14ac:dyDescent="0.35">
       <c r="O80" s="3" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="81" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="81" x14ac:dyDescent="0.35">
       <c r="O81" s="3" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="82" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="82" x14ac:dyDescent="0.35">
       <c r="O82" s="3" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="83" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="83" x14ac:dyDescent="0.35">
       <c r="O83" s="3" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="84" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="84" x14ac:dyDescent="0.35">
       <c r="O84" s="3" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="85" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="85" x14ac:dyDescent="0.35">
       <c r="O85" s="3" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="86" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="86" x14ac:dyDescent="0.35">
       <c r="O86" s="3" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="87" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="87" x14ac:dyDescent="0.35">
       <c r="O87" s="3" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="88" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="88" x14ac:dyDescent="0.35">
       <c r="O88" s="3" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="89" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="89" x14ac:dyDescent="0.35">
       <c r="O89" s="3" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="90" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="90" x14ac:dyDescent="0.35">
       <c r="O90" s="3" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="91" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="91" x14ac:dyDescent="0.35">
       <c r="O91" s="3" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="92" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="92" x14ac:dyDescent="0.35">
       <c r="O92" s="3" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="93" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="93" x14ac:dyDescent="0.35">
       <c r="O93" s="3" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="94" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="94" x14ac:dyDescent="0.35">
       <c r="O94" s="3" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="95" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="95" x14ac:dyDescent="0.35">
       <c r="O95" s="3" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="96" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="96" x14ac:dyDescent="0.35">
       <c r="O96" s="3" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="97" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="97" x14ac:dyDescent="0.35">
       <c r="O97" s="3" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="98" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="98" x14ac:dyDescent="0.35">
       <c r="O98" s="3" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="99" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="99" x14ac:dyDescent="0.35">
       <c r="O99" s="3" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="100" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="100" x14ac:dyDescent="0.35">
       <c r="O100" s="3" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="101" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="101" x14ac:dyDescent="0.35">
       <c r="O101" s="3" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="102" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="102" x14ac:dyDescent="0.35">
       <c r="O102" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="103" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="103" x14ac:dyDescent="0.35">
       <c r="O103" s="3" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="104" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="104" x14ac:dyDescent="0.35">
       <c r="O104" s="3" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="105" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="105" x14ac:dyDescent="0.35">
       <c r="O105" s="3" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="106" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="106" x14ac:dyDescent="0.35">
       <c r="O106" s="3" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="107" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="107" x14ac:dyDescent="0.35">
       <c r="O107" s="3" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="108" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="108" x14ac:dyDescent="0.35">
       <c r="O108" s="3" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="109" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="109" x14ac:dyDescent="0.35">
       <c r="O109" s="3" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="110" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="110" x14ac:dyDescent="0.35">
       <c r="O110" s="3" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="111" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="111" x14ac:dyDescent="0.35">
       <c r="O111" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="112" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="112" x14ac:dyDescent="0.35">
       <c r="O112" s="3" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="113" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="113" x14ac:dyDescent="0.35">
       <c r="O113" s="3" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="114" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="114" x14ac:dyDescent="0.35">
       <c r="O114" s="3" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="115" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="115" x14ac:dyDescent="0.35">
       <c r="O115" s="3" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="116" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="116" x14ac:dyDescent="0.35">
       <c r="O116" s="3" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="117" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="117" x14ac:dyDescent="0.35">
       <c r="O117" s="3" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="118" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="118" x14ac:dyDescent="0.35">
       <c r="O118" s="3" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="119" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="119" x14ac:dyDescent="0.35">
       <c r="O119" s="3" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="120" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="120" x14ac:dyDescent="0.35">
       <c r="O120" s="3" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="121" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="121" x14ac:dyDescent="0.35">
       <c r="O121" s="3" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="122" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="122" x14ac:dyDescent="0.35">
       <c r="O122" s="3" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="123" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="123" x14ac:dyDescent="0.35">
       <c r="O123" s="3" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="124" spans="15:15" x14ac:dyDescent="0.4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="124" x14ac:dyDescent="0.35">
       <c r="O124" s="3" t="s">
         <v>94</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AK124" xr:uid="{2C3D481A-1F78-43FC-A96C-7E83E3560056}"/>
+  <autoFilter ref="A1:AK124"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -11006,6 +11008,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E033184CEB11F648BBD0F70F1BE6A53E" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6772e668bd11b5d68af2caf9f3d3ff0e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="a44a327f-4c77-4059-bb07-e278862d87fb" xmlns:ns4="7fa3c9fb-ef78-47d6-a04f-8ab7fe78f626" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d1370a7ae997dfead2b2ac8f1c36ed42" ns3:_="" ns4:_="">
     <xsd:import namespace="a44a327f-4c77-4059-bb07-e278862d87fb"/>
@@ -11228,22 +11245,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EE1F3C90-AF98-43AB-B3C2-ECE16BFEAB58}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="a44a327f-4c77-4059-bb07-e278862d87fb"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="7fa3c9fb-ef78-47d6-a04f-8ab7fe78f626"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA715A9A-50E5-49B3-81AC-118F4B5A14E8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4BE07B4-EAD3-43BB-A412-78B98636CC41}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11260,29 +11287,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA715A9A-50E5-49B3-81AC-118F4B5A14E8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EE1F3C90-AF98-43AB-B3C2-ECE16BFEAB58}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="a44a327f-4c77-4059-bb07-e278862d87fb"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="7fa3c9fb-ef78-47d6-a04f-8ab7fe78f626"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>